<commit_message>
Loop iter 2: Sources & Uses block + EBITDA bridge (Y1->Y3)
- Dashboard S&U (close through refi): $750K sources (250 equity + 500 refi) =
  $125K down + $380.6K seller payoff (incl $5.6K accrued int) + $244.4K net WC
  retained; residual-positive check wired to conventions
- EBITDA bridge Y1->Y3: $263K + $728K volume + $222K rate/margin - $237K overhead
  growth = $976K (ties to actual, check = 0)
- Fixed missing sheet prefix in S&U SUMPRODUCT (was reading Dashboard rows)
QA 20/20. All P0/P1 items from the PE research checklist now implemented.

https://claude.ai/code/session_01GAHLyfqLR9bxwN2jm6VjPU
</commit_message>
<xml_diff>
--- a/financial_models/output/Azalea_Hospice_Proforma_Rev3.00_DYNAMIC.xlsx
+++ b/financial_models/output/Azalea_Hospice_Proforma_Rev3.00_DYNAMIC.xlsx
@@ -2052,7 +2052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL27"/>
+  <dimension ref="A1:AL45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5298,8 +5298,178 @@
         <v/>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>SOURCES &amp; USES (close through refinance month)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Sources: equity on deposit</t>
+        </is>
+      </c>
+      <c r="B30" s="22">
+        <f>'Control Tower'!$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sources: refinance note proceeds</t>
+        </is>
+      </c>
+      <c r="B31" s="22">
+        <f>IF('Control Tower'!$B$16=1,'Control Tower'!$B$18,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL SOURCES</t>
+        </is>
+      </c>
+      <c r="B32" s="23">
+        <f>B30+B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Uses: down payment at close</t>
+        </is>
+      </c>
+      <c r="B33" s="22">
+        <f>'Control Tower'!$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Uses: seller payoff at refi (principal + accrued interest)</t>
+        </is>
+      </c>
+      <c r="B34" s="22">
+        <f>IF('Control Tower'!$B$16=1,SUMPRODUCT(('Cash Flow &amp; Runway'!$C$4:$AL$4='Control Tower'!$B$17)*('Cash Flow &amp; Runway'!$C$14:$AL$14+'Cash Flow &amp; Runway'!$C$15:$AL$15)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Uses: pre-opening / startup spend</t>
+        </is>
+      </c>
+      <c r="B35" s="22">
+        <f>'Control Tower'!$B$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Uses: net working capital retained (residual)</t>
+        </is>
+      </c>
+      <c r="B36" s="23">
+        <f>B32-B33-B34-B35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>CHECK: sources - uses = 0 by construction; residual must be &gt; 0</t>
+        </is>
+      </c>
+      <c r="B37" s="21">
+        <f>IF(B36&gt;0,0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>EBITDA BRIDGE - Year 1 to Year 3 (attribution walk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Year 1 EBITDA</t>
+        </is>
+      </c>
+      <c r="B40" s="23">
+        <f>SUM('P&amp;L'!C24:N24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>+ Census / volume effect (added PDs at Y1 contribution/PD)</t>
+        </is>
+      </c>
+      <c r="B41" s="22">
+        <f>(SUM('Census Waterfall'!AA12:AL12)-SUM('Census Waterfall'!C12:N12))*(SUM('P&amp;L'!C15:N15)/SUM('Census Waterfall'!C12:N12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>+ Rate / margin-per-PD effect (Y3 PDs x change in contribution/PD)</t>
+        </is>
+      </c>
+      <c r="B42" s="22">
+        <f>SUM('Census Waterfall'!AA12:AL12)*(SUM('P&amp;L'!AA15:AL15)/SUM('Census Waterfall'!AA12:AL12)-SUM('P&amp;L'!C15:N15)/SUM('Census Waterfall'!C12:N12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>- Overhead growth (indirect labor + facility + G&amp;A)</t>
+        </is>
+      </c>
+      <c r="B43" s="22">
+        <f>-((SUM('Staffing'!AA38:AL38)+SUM('Operating Budget'!AA18:AL18)+SUM('Operating Budget'!AA31:AL31))-(SUM('Staffing'!C38:N38)+SUM('Operating Budget'!C18:N18)+SUM('Operating Budget'!C31:N31)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>Year 3 EBITDA (bridge total)</t>
+        </is>
+      </c>
+      <c r="B44" s="23">
+        <f>B40+B41+B42+B43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Year 3 EBITDA (actual, tie check = 0)</t>
+        </is>
+      </c>
+      <c r="B45" s="22">
+        <f>SUM('P&amp;L'!AA24:AL24)-B44</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A39:D39"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>